<commit_message>
Passaggio forzato a Gemini 1.5 Flash-8B per gestione quota
</commit_message>
<xml_diff>
--- a/Risultati/Geopolitica.xlsx
+++ b/Risultati/Geopolitica.xlsx
@@ -458,270 +458,270 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sovranità economica e geopolitica: il ruolo dell’Europa tra Stati Uniti e Cina - Confcommercio</t>
+          <t>Adeguati assetti, come la geopolitica cambia le architetture socio-tecniche d’impresa - Agenda Digitale</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sovranità economica e geopolitica: il ruolo dell’Europa tra Stati Uniti e Cina  Confcommercio</t>
+          <t>Adeguati assetti, come la geopolitica cambia le architetture socio-tecniche d’impresa  Agenda Digitale</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tue, 14 Apr 2026 15:38:31 GMT</t>
+          <t>Thu, 23 Apr 2026 13:36:53 GMT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiYEFVX3lxTE1tN285RW9PWUEwWmhJTEFXSDY0c01mR1Q1UTRuVXdvQUVGeVYzdzQ0a2EyV2cxand5Z01USF9xUzh2VWtHMW9qNjRrRnpNQ3M3bmNiTDhUQnhlMjVCTEJjRg?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQblpBQzF3NGJJZ1FxZ2g5WVh0TE1MckFyaWJFb2pHTXlyeld0UGwwbmZ6TjF2dlc2N3RIeTZnZjVxcFFqWnR0RV9DNHFWUmlzcEJFcmtmaHNVMGF1QWJVNnhmMTRHbEdwMEZPNDZ0MktkT09kZmg4UEhJNDlMWkFkVHplY01sV3k0cHZFQVBEaWJwQ1JnWFBfMlBkbXhDRFlsTDJRZTFrdVpSY2djTng1TGt2ODZ4cnBFLU5HQndDcDVzUQ?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>{'href': 'https://www.confcommercio.it', 'title': 'Confcommercio'}</t>
+          <t>{'href': 'https://www.agendadigitale.eu', 'title': 'Agenda Digitale'}</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Draghi: "Fine delle regole globali, il commercio è ormai guidato dalla geopolitica" - Video - Adnkronos</t>
+          <t>L’Artico al centro del mondo: tra geopolitica e avventura al Mercato Centrale Torino - mercatocentrale.it</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Draghi: "Fine delle regole globali, il commercio è ormai guidato dalla geopolitica" - Video  Adnkronos</t>
+          <t>L’Artico al centro del mondo: tra geopolitica e avventura al Mercato Centrale Torino  mercatocentrale.it</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wed, 15 Apr 2026 14:25:00 GMT</t>
+          <t>Wed, 22 Apr 2026 16:38:34 GMT</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNN1hRcEpPUFNkZUtQSFc4SFJuU1FDRUlMd25hd05jZC1yQnBXdFEzUGhxYTUxTTUtUkxKZ1FUbVk4a3h1QW9RVEgtaGREMEtXa2hBVnFYeGo2QTFLTDNHbGJoV3Y1MVd1Q0FKWnNPUkVxcEV3ajRZSkFIN1lSb1lsWXpTVFNmQm9KZVJWaGp6ZC1ZVTB6U2JOOU52d0F5UTM0a3JuN21wYjBYX2xXM1EwOU1HQ3RkbDgwTGtSTjc4V1ZFaDFIMk1QRlh5WTRhZ2tqeUdF?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOdWVoNnZva253T1BXZ29MNEgwcHJPOE1vTm1PREhRdDBKOHhsQjFfN1lEMjdUaDlmd3pyaVZvZ2N0bWVSaW9OOUVKNjZjek9BX0dPaTF2N2otMDRjbnM4bHpiR0R2TURPVGw4V1VuOG9oQUtmY0lKT3RDWHprM2ltd3M1TEozMXc3MnE5S09HR3E1aEE3VmpJNUh6N21rRHI2WFpBTTZSMU1YcDNQMTdzbFlWLWU0RWtFRlQ0?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>{'href': 'https://www.adnkronos.com', 'title': 'Adnkronos'}</t>
+          <t>{'href': 'https://www.mercatocentrale.it', 'title': 'mercatocentrale.it'}</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Geopolitica delle narrazioni e riformismo erosivo: la strategia globale della Cina - L'Eurispes</t>
+          <t>Geopolitica e giovani protagonisti del Festival di Trento - Il Sole 24 ORE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Geopolitica delle narrazioni e riformismo erosivo: la strategia globale della Cina  L'Eurispes</t>
+          <t>Geopolitica e giovani protagonisti del Festival di Trento  Il Sole 24 ORE</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thu, 16 Apr 2026 10:06:44 GMT</t>
+          <t>Mon, 20 Apr 2026 17:56:29 GMT</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOZElpSUU2dWlTWnZIQXFRTDFNWVA1WDBxU3ZZSzFOVHBCeEd0ZW56dmhGZDNON1g1dVBLZHRodmVJZ2tiZlNaaVlUbVhTNDJoRXp1eUxYU3Voenh3dlZMTzFETDFaSWJGQXp5M3ppcGNWTjQzc3kyR0VvYzZ2QVktS1J6em9HN2wxc0ZMVXhwUQ?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPN3lxZERDSDlrTnlVWV9YRzkySERlMDBqU2hFTmJybWxKU29CaDBCejF2WDZ2Q1FhZHBWbFMxbUphR1lVRWVNSUxqZGdjVWVuQ0d1NERETFYzVHp2c3pKMk8wRTE3Nk9FNnNqY0hzb3UtSVg2MG5mejVHdHIxaUJJaWd3Y2lycjZEQjNuZ2hGZk5Cal9VVnc?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>{'href': 'https://www.leurispes.it', 'title': "L'Eurispes"}</t>
+          <t>{'href': 'https://www.ilsole24ore.com', 'title': 'Il Sole 24 ORE'}</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Geopolitica, come le telco possono costruire una nuova resilienza tecnologica - CorCom</t>
+          <t>Governare l’incertezza: perché serve una nuova classe dirigente - Geopolitica.info</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Geopolitica, come le telco possono costruire una nuova resilienza tecnologica  CorCom</t>
+          <t>Governare l’incertezza: perché serve una nuova classe dirigente  Geopolitica.info</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tue, 14 Apr 2026 08:08:01 GMT</t>
+          <t>Thu, 23 Apr 2026 07:22:06 GMT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxORTJNdW1EMjlJV3JTelFRdkZoZUtlZUVWWGx2WFljT0dfRkNBMXVRNWFJQXp4SDI3ZmZ5bUJSRTBjLVg4aWIwU04xczJDUnBiaGt3T0QzbDQzMG00UURxUmtJNEdBTXNSWjE1MVVpOXRCd0JhcWhfWHFVWmtTVDB0LXh0ZWZJX1cyOWhEUndYVl9keDZMNlJrQkV6bEs5TVdQMTVjLUtLZHpkMWlBbnBQbTdyWWxocmk3VVFmcEdYSkt2X25LM1R0ZA?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFBCUEtTRDgxUTY2SFAySUw3TVFXamxvS0dENnQ0b0tDdFJFNGdGVEM1Z0dWTTNmUU1RVEs2Z0NuMTBRRjdfVEdTUVZ6NVM2SV9VZGpYMFJsVmJRRktxd1ZnZ24zY21xMlZWOTRaMFRnanM?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>{'href': 'https://www.corrierecomunicazioni.it', 'title': 'CorCom'}</t>
+          <t>{'href': 'https://geopolitica.info', 'title': 'Geopolitica.info'}</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CGIA E CIRCOLO VENETO: COMUNITA’ GEOPOLITICA E DIFESA – giovedì 16 aprile 2026 – Novotel Mestre - CGIA mestre</t>
+          <t>Corea del Sud, il rally azionario che sfida la geopolitica - FocusRisparmio</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CGIA E CIRCOLO VENETO: COMUNITA’ GEOPOLITICA E DIFESA – giovedì 16 aprile 2026 – Novotel Mestre  CGIA mestre</t>
+          <t>Corea del Sud, il rally azionario che sfida la geopolitica  FocusRisparmio</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Thu, 16 Apr 2026 15:13:24 GMT</t>
+          <t>Mon, 20 Apr 2026 05:41:08 GMT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOY2t0WHI3RVNwS0JGUnB5a3RBaGwzUzFDRk5CaWVOTG12WTlpNjJmdlF5QnBGcmlQbjZIQzdYdHlGWnRjMHNOOTFQeUlkdlo3T0tjWllQUl8zZTBoT01LT05fd2UzbEZkUm9Wajl0OU1OQVJ4aG1EWnIxMnVNbEhDWjJDTjUyS1JVckpzWDZwb0hrY2x4eVRnT1JRZG9YSEJNdHppYmRoSmVtRVUwa29mVkxqSmtTV2hXNnFj?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOTzQ3Q0ZVQzRVaTRla0kzNjZ4UzVqbVZrZ3lMVGFMUEphOUUxT1FhRk4xY2VweGJVdlZGMS1oVEt4cXBVaDZWMWV0azNYWVFNSldCb3Rhc3B2U3lOLWJlNDJBZ0pjdTRfbVpGa2V0T0RidGxfeG8xRm1JMzdtd0xLTFRkUzhGQ094RDB2SHdSdll0VWNHYWc?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>{'href': 'https://www.cgiamestre.com', 'title': 'CGIA mestre'}</t>
+          <t>{'href': 'https://www.focusrisparmio.com', 'title': 'FocusRisparmio'}</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Geopolitica e riforme normative a Pechino spingono i mercati azionari asiatici - MarketScreener Italia</t>
+          <t>La geopolitica dei poliamori e la solitudine delle persone - Corriere della Sera</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Geopolitica e riforme normative a Pechino spingono i mercati azionari asiatici  MarketScreener Italia</t>
+          <t>La geopolitica dei poliamori e la solitudine delle persone  Corriere della Sera</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Mon, 20 Apr 2026 10:43:29 GMT</t>
+          <t>Fri, 24 Apr 2026 06:04:00 GMT</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOT3ZaYXk5RlhqME9jQnFpSHFwdUJYUFdtaUd6YTNqdWxnSGNJV1FHUTR0dTJTTWZJTE9fVmI1MzdGd05jb3Uyc2p4V3FMODRqNjJSTll1TDNCWUhPM0lTT2FQZ29WWTdWN2hOYlFncC1LeVpmWVhsQmt5TW51ZXNQTzJSSVk5VjNuWFlIUGVWb2xRbTV6ZEU1c05kakJubXQ5S0xDYXp4TEx4eXNKN2JXc0E2RVNYektLajV5em9wRkJXZFFyYncyb05wSzNpZw?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxOX0tGc0YtbUJjVW42VE1pSHZ1UW85YlpkZ0VUYklqN3lkLUY2TXBVMUpSQjJzaVpFZ290bHB1ZHRERVFKVlYzcl9razJ1c1NTY1ZLTlJxZDVQU2hkY29CMFZJNkpfMFhpcTZST3hOSHFRWS1wMWlNVnZod2h5UFgwRkhPcjI1aXh0ZFhRbkRvOWt4SjZZaDhGSWVxcVhMNWJ2bUNSZmdPamxyWEZsQ3BWclhKczlrNi1ZS2l5a1YyY05vSmd5Q01ySF9ySUNUMTExRVAySzRJdEhnMWdr?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>{'href': 'https://it.marketscreener.com', 'title': 'MarketScreener Italia'}</t>
+          <t>{'href': 'https://www.corriere.it', 'title': 'Corriere della Sera'}</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Geopolitica e mercati, Vedda (DWS): “Volatilità elevata ma lo scenario resta costruttivo” - FocusRisparmio</t>
+          <t>Geopolitica al centro: il nuovo AMC sui grandi trend globali - Websim</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Geopolitica e mercati, Vedda (DWS): “Volatilità elevata ma lo scenario resta costruttivo”  FocusRisparmio</t>
+          <t>Geopolitica al centro: il nuovo AMC sui grandi trend globali  Websim</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wed, 15 Apr 2026 11:11:15 GMT</t>
+          <t>Fri, 24 Apr 2026 12:00:00 GMT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxQdlRENzk5WEZESUR3TkVOMUJxQ3FmOFR1R0pTLWdsSlN1cC1qdDRLYUVhTFpqZHlRQkdOVW9VU2QwYkhqOEJMNG81UUlyRWxHeFVtQVJSOVlTYm1mNzAtWDdlcXhCam9DWFBCNlF5bFNLMENsbjhxRF9Pc1RuZmJ6N01oTEp1anF2TzVpVUlpZ2RFS1owSlVkclVaRDdPSmQtcWVtNFN2YnhOUWtqTWc?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNZmFRMmhVN1BhazdvQlg4Y3lMekhwc0NaeTdQdjd6ajU2VUdfYmp5cXN3elAzR2NNaWJSNGpDSTVEVVZIZE5JQV9DU1EyZTVHTkFSaVI0QkpKVTZFMGlHSDFkVmVzNnphbV9jUk51Zm1Wb3NmdE1LaUxNTXM1N2lFWXEwdWZSNkVadGxvM3pEV094bUxYcHlJM1kzX2pUUFZqdG5kZzBoXzdrRS1VX0p6ZVBrX2Q?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>{'href': 'https://www.focusrisparmio.com', 'title': 'FocusRisparmio'}</t>
+          <t>{'href': 'https://www.websim.it', 'title': 'Websim'}</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sistemi di conflitto intersecati nel Corno d’Africa: rischi di guerra regionale e ricadute globali - Geopolitica.info</t>
+          <t>L’Italia, la geopolitica e le scelte obbligate. O no - Sky TG24</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Sistemi di conflitto intersecati nel Corno d’Africa: rischi di guerra regionale e ricadute globali  Geopolitica.info</t>
+          <t>L’Italia, la geopolitica e le scelte obbligate. O no  Sky TG24</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fri, 17 Apr 2026 10:57:16 GMT</t>
+          <t>Sat, 18 Apr 2026 12:13:22 GMT</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNbHZzT1d0Y2tkVjh2ZjQxV3RZN21PbmZ5NmRDYWN2Tm8wX2xiNUNVZFViMFBjZkU5WWxsUFNaNU9OUllMZUNrTHVuaXFoTmVJWXptYjc2SjNYT1VMbGNjMUFQczBDTGxlbzN5ZEU4UWQ0M1FERjRwcHh4WmNsejFFVkZSZ0JuZmphTDFsTnh2d0JhYmhFWVNHTGt5cTdmbHphcHFUMlYyZG9Ua0szMUpwNERXTTlPSERaZmxBcXNocw?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBNTV9MYmZXZTV4V1R4Q2VCcVhLc0REUG42U2d1NHNVN19yNTRuS0c5cTZ2WmJYR2ZxcmxYUGFJOHFYcnNFQS1uMzRMRFIyUGpMOFlsVHBxZ2NfakU3QkR4TEc3RWRKbE1IMmRB?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>{'href': 'https://geopolitica.info', 'title': 'Geopolitica.info'}</t>
+          <t>{'href': 'https://tg24.sky.it', 'title': 'Sky TG24'}</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Rassegna di Geopolitica. Dopo il fallimento dei colloqui,Trum annuncia un blocco navale americano nello Strett - Radio Radicale</t>
+          <t>Scommesse da 760 milioni sul petrolio all’ombra di Gekko: la geopolitica di Trump è un insider trading globale? - Corriere del Ticino</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Rassegna di Geopolitica. Dopo il fallimento dei colloqui,Trum annuncia un blocco navale americano nello Strett  Radio Radicale</t>
+          <t>Scommesse da 760 milioni sul petrolio all’ombra di Gekko: la geopolitica di Trump è un insider trading globale?  Corriere del Ticino</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sat, 18 Apr 2026 05:00:00 GMT</t>
+          <t>Mon, 20 Apr 2026 18:37:00 GMT</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxPTy1mU2otamhhR2k5eFBhUktvSDdETTlrZzBmRFhHSG1kbTZ1NWtSQW9KTmRYdkxDQWFjbHlJOHZzbm1WTDRTUU16OHVBTVhYcGtKcnhCckVsUEpMbVJKaExucXUzWnl2VW5LY0lCcUI0bmNFc3d4UldOd3dFUFRWTEpIVWZFNU9GN3VpSTFxMmwwN1huYlRZYXVjTlRiaTNsMWM4UmlDNGVfNFE4SlY0Uk5MeXNwTnJ5eGxwNWM4d0paeFQ4NlZv?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxQNlluRWM4UGRiUlNYWnhYTXZNMDl1R0lZakxaNnpBQldwU1I1WjBmMWJDY3NuaFhzSjZ3MXRwdjBWdnJENjg1Ny1VYXNKaXFUcjVaWk91VWZMXy1xVzk2cUNyeWtRYm9GOFd2emJLNWptcUJHSmZaZ2ZGT01Ya1ZGc0UwaEVnYkdkeEVxcEhwZ1VOTlhZdGZ4Y091SmZoaU01QldQLU5nVFE2VktZeHEtWWQ3MThhU2d6YVFkR1BqcnhXZm9zV1VNVE1NdlRIYzZpZmVNeFUxYktKTGJzalI3Q0VrMHNuMFVLanc?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>{'href': 'https://www.radioradicale.it', 'title': 'Radio Radicale'}</t>
+          <t>{'href': 'https://www.cdt.ch', 'title': 'Corriere del Ticino'}</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Crisi geopolitica e oro: un equilibrio precario - Milano Finanza</t>
+          <t>La pressione geopolitica sui prezzi colpisce il mercato dei fertilizzanti e dei ritardanti di fiamma - chemeurope.com</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Crisi geopolitica e oro: un equilibrio precario  Milano Finanza</t>
+          <t>La pressione geopolitica sui prezzi colpisce il mercato dei fertilizzanti e dei ritardanti di fiamma  chemeurope.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wed, 15 Apr 2026 07:00:00 GMT</t>
+          <t>Fri, 24 Apr 2026 01:10:44 GMT</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPQjB2TlNTaXZXRE9zeXlJSWZJZV9DYUdhV1JTZUcwRzE5LVVCd00zLUdQeUQwNjZONkRPZFdkY0t6amJVUlpwN0RIc1lfTUtuNG5TZk9EaDFTTk04OW9KSlNJdG81YW1QMUtEZEJmSXRycTg3aGF0cnExQWQtMU5iM1RhdXVJWGpyUDIwNkQ2T3JULUlwcm5EYnY5bmdLUkpKdkxreVlHVU8tM0ZoUkI5MWNZeVM5UQ?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
+          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxPd0R1XzFJZHlORWYwc0RSOFh1RVRsQ2lGcHVBUmFjWjhJa1h6Nk1wX1ZrSE5mSjhNWmhWRERxZjZKSkxqT3l1Mnd5MUhhRkNDY1RJcW05dEpMM05BdmJ2S2pkOU94ZmtoZ3BkN2RETlRRVG5NT2VvTS1WU19sdnFhRjJqdFVrdEZsZVh3Znk1VUp3dW5PaDcyWU1qaUJvenAwQTBKbnZaTGRBNUxfbWFnVTlxdDctRm95bW5HZG91STVTeDJ1MlRJaGd2OFFRSnFYUG9Uck5QTzlET1pXQzZXdnl3dlZoQQ?oc=5&amp;hl=en-US&amp;gl=US&amp;ceid=US:en</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>{'href': 'https://www.milanofinanza.it', 'title': 'Milano Finanza'}</t>
+          <t>{'href': 'https://www.chemeurope.com', 'title': 'chemeurope.com'}</t>
         </is>
       </c>
     </row>

</xml_diff>